<commit_message>
Spell monitor panel, GPU fallback, 4-part versions released on demand
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -6656,7 +6656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7748,6 +7748,151 @@
       </c>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>SM-01</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>[แผงติดตาม] ว่าง</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>เปิดแท็บคิวแก้ไขตอนไม่มีงานตรวจ</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้น "⏸ ระบบตรวจคำผิดว่าง" และปุ่ม "ตรวจคำผิดทั้งคิว" · ถ้าวันนี้เคยตรวจแล้วมีบรรทัดสถิติ "วันนี้ตรวจแล้ว N ตอน · เฉลี่ย … · GPU ใช้ไป x/300 วิ"</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>SM-02</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>[แผงติดตาม] กำลังตรวจ</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>สั่งตรวจทั้งคิว แล้วดูแผง</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้นโหมด (⚡ GPU หรือ CPU) · "กำลังตรวจ: ชื่อตอน · ส่วนที่ i/n · เวลาที่ใช้" พร้อมแถบความคืบหน้าที่ขยับตามส่วน · "รอคิว N ตอน · เหลือราว M นาที" · ตัวเลขอัปเดตเองทุก ~5 วิ</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>SM-03</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>[GPU] โหมดเร่งความเร็ว</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>ตรวจตอนแรกของวัน (ยังมีโควต้า GPU)</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>แผงขึ้น "⚡ โหมดเร่งความเร็ว (GPU)" · ตรวจเสร็จเร็วกว่าเดิมชัดเจน (เดิม ~2 นาที/ตอน) · สถิติ GPU ใช้ไปเพิ่มขึ้น</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>SM-04</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>[GPU] โควต้าหมด</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>ตรวจหลายตอนจนโควต้า GPU วันนี้หมด</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>ไม่มี error · แผงเปลี่ยนเป็น "โหมดปกติ (CPU)" + "โควต้า GPU วันนี้หมด · ลองเร่งความเร็วอีกครั้ง HH:MM" · ตรวจต่อจนครบ (ช้าลง)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>SM-05</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>[แผงติดตาม] งานของโปรเจกต์อื่น</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>ระหว่างที่มีงานตรวจของอีกโปรเจกต์/ผู้ใช้อื่น เปิดคิวแก้ไขของโปรเจกต์นี้</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้น "กำลังตรวจ: ตอนจากโปรเจกต์อื่น" · "รอคิว N ตอน (ของโปรเจกต์นี้ K)" · ไม่เห็นชื่อตอนของคนอื่น · ปุ่มหยุดถอนได้เฉพาะของโปรเจกต์นี้</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deeper plot threads: summary, issues, parent/links, tension
- Schema: plot_threads.summary + parent_thread_id, new plot_thread_points and
  plot_thread_links tables, plot_thread_beats.point_id + tension
- Server actions for points, links, beat updates; parent cycle guard
- Network warnings (resolve order, decoy, open issues after payoff, flat tension)
  with a check wired into npm run check
- Thread ledger UI: expandable details, issue checklist, tension dots + sparkline

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -27,6 +27,7 @@
     <sheet name="เลนบนกระดาน v2.8.0" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="เส้นเชื่อมสีล้วน v2.10.0" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="ตรวจคำผิด v2.12.0" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="ปมเชิงลึก (ใหม่)" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ผู้ช่วย AI (ใหม่)'!$A$1:$G$19</definedName>
@@ -546,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -741,6 +742,16 @@
         <is>
           <t>24</t>
         </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>ปมเชิงลึก (ใหม่)</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -8189,6 +8200,704 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>PT-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>[รายละเอียด] เปิด/ปิด</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>เปิดสมุดปม กดลูกศรหน้าชื่อปม แล้วกดอีกครั้ง</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>กดครั้งแรกกางแผงคำอธิบาย/ประเด็น/อยู่ใต้ปม/ความสัมพันธ์ · ลูกศรหมุนลง · กดซ้ำย่อกลับ</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>PT-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>[คำอธิบาย] บันทึก</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>กางปม พิมพ์ในช่อง "ปมนี้คืออะไร" แล้วคลิกนอกช่อง → ปิดสมุดแล้วเปิดใหม่</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ข้อความยังอยู่ · ตอนย่อปมเห็นตัวอย่างคำอธิบาย 2 บรรทัดใต้ชื่อ</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>PT-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>[คำอธิบาย] ไม่แก้ไม่บันทึก</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>คลิกเข้า-ออกช่องคำอธิบายโดยไม่พิมพ์อะไร</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ไม่มี toast error · ไม่มีการโหลดซ้ำที่สังเกตได้</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>PT-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>[ประเด็น] เพิ่ม</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>พิมพ์ประเด็นแล้วกด Enter (และอีกข้อกดปุ่ม +)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ประเด็นขึ้นเรียงตามลำดับที่เพิ่ม · ช่องว่างลง · หัวปมขึ้น "ประเด็น 0/2"</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>PT-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>[ประเด็น] ช่องว่าง</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>กด Enter ตอนช่องว่าง หรือมีแต่เว้นวรรค</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ไม่เพิ่มประเด็น · ปุ่ม + กดไม่ได้</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>PT-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>[ประเด็น] ติ๊กคลี่แล้ว</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>กดวงกลมหน้าประเด็น แล้วกดซ้ำ</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>กดครั้งแรก: ไอคอนติ๊กเขียว ข้อความขีดฆ่า ตัวนับเป็น 1/2 · กดซ้ำกลับเป็นเปิด</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>PT-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>[ประเด็น] ลบ</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ชี้ที่ประเด็นที่มีฉากเลือกไว้ กด X</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>ประเด็นหาย · ฉากที่เคยเลือกประเด็นนั้นกลับเป็น "— ประเด็น —" ไม่ error</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>PT-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>[ฉาก] เลือกประเด็น</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>กางปมที่มีประเด็นและผูกฉากแล้ว เลือกประเด็นในดรอปดาวน์ข้างฉาก แล้วย่อปม</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>ตอนย่อ ชื่อฉากต่อท้ายด้วย " · &lt;ประเด็น&gt;" · ปมที่ไม่มีประเด็นไม่โชว์ดรอปดาวน์</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>PT-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>[ความตึง] ให้คะแนน</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>กดจุดที่ 3 ข้างฉาก แล้วกดจุดที่ 3 ซ้ำ</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>กดแรก: จุด 1-3 เป็นสีส้ม · กดซ้ำ: ล้างเป็นเทาหมด</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>PT-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>[ความตึง] เส้นกราฟ</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>ให้คะแนนอย่างน้อย 2 ฉากในปมเดียว</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>เส้นกราฟเล็กโผล่ใต้หัวปม ขึ้นลงตามคะแนน · มีคะแนนฉากเดียวไม่โชว์เส้น</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>PT-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>[เตือน] ความตึงไม่เพิ่ม</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่ฉากบทต้นได้ 4 และฉากบทหลังได้ 2 (ฉากต้องผูกบทแล้ว)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้นป้าย "ความตึงไม่เพิ่มขึ้น" (สีเทา) · ปรับฉากหลังเป็น 5 แล้วป้ายหาย</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>PT-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>[ปมแม่] ตั้ง</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ปม B เลือก "อยู่ใต้ปม" = A</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>B ย้ายไปอยู่ใต้ A ย่อหน้าเยื้องและมีไอคอนต้นไม้</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>PT-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>[ปมแม่] กันวน</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>หลังทำ PT-12 กางปม A เปิดดรอปดาวน์ "อยู่ใต้ปม"</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ไม่มี A เอง และไม่มี B (ลูกของ A) ให้เลือก</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>PT-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>[ปมแม่] ลบแม่</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>ลบปม A ที่มี B เป็นลูก</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>B ยังอยู่ ขึ้นมาเป็นปมระดับบน ไม่เยื้อง</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>PT-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>[ความสัมพันธ์] ต้องเฉลยก่อน</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>ปม A เพิ่มความสัมพันธ์ "ต้องเฉลยก่อน" B · ใส่ฉากเฉลยของ B ที่บท 3 · ยังไม่ให้ A เฉลย</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>A ขึ้นป้ายส้ม "ต้องเฉลยก่อน "B" แต่ช้ากว่า" · ปุ่มสมุดปมนับเตือนเพิ่ม</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>PT-16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>[ความสัมพันธ์] ลำดับถูก</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>ต่อจาก PT-15 ใส่ฉากเฉลยของ A ที่บท 2 (หรือบทเดียวกับ B)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>ป้ายเตือนลำดับหาย</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>PT-17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>[ความสัมพันธ์] ปมหลอก</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>ปม D "เป็นปมหลอกของ" B · B เฉลยแล้ว · D ยังไม่เฉลย</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>D ขึ้น "ปมหลอกยังไม่คลี่ ทั้งที่ "B" เฉลยแล้ว" · ตั้งสถานะ D เป็น "ตั้งใจทิ้ง" แล้วป้ายหาย</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>PT-18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>[ความสัมพันธ์] ซ้ำ/ลบ</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>เพิ่มความสัมพันธ์เดิมซ้ำ แล้วกด X ลบ</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>ไม่เกิดแถวซ้ำ ไม่ error · ลบแล้วแถวหาย</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>PT-19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>[เตือน] เฉลยแต่ประเด็นค้าง</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่มีประเด็นเปิดอยู่ 1 ข้อ ตั้งสถานะ "เฉลยแล้ว"</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้น "เฉลยแล้ว แต่ประเด็นค้าง 1 ข้อ" · ติ๊กประเด็นแล้วป้ายหาย</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>PT-20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>[ของเดิม] ปมเก่า</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>เปิดปมที่สร้างก่อนรอบนี้</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>แสดงปกติ คำอธิบาย/ประเด็นว่าง ไม่มีคำเตือนใหม่ผุดขึ้นเอง · เตือนเดิม (ยังไม่เฉลย/ไม่ถูกแตะ) ยังทำงาน</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>PT-21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>[ของเดิม] ผูกปมจากการ์ด</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>บน playground ผูกปมกับการ์ด และสร้างปมใหม่จากการ์ด</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>ทำงานเหมือนเดิม ไม่ error · ปมใหม่โผล่ในสมุดปม</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>PT-22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>[ข้อจำกัด] ลบแล้วย้อนกลับ</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>ลบปมที่มีคำอธิบาย/ประเด็น แล้วกด "ย้อนกลับ" ใน toast</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>ปมกลับมาพร้อมฉากที่ผูก แต่คำอธิบาย/ประเด็น/ความสัมพันธ์/ความตึงหาย (ข้อจำกัดที่รู้แล้ว task.md ข้อ 18)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Threads tab two-pane layout; split thread status into progress + intent
- Threads tab: list on the left, selected thread detail on the right;
  selection kept in ?thread=, single pane on narrow screens
- Progress (unseeded/seeded/developing/partial/paid) is now computed from
  scenes and issues; status column holds author intent
  (active/on_hold/open_ended/abandoned), legacy values read as active
- New optional target chapter per thread with an overdue warning
- addBeat no longer auto-sets status to paid; chapter report, thread ribbon
  and story-format share threadNeedsPayoff

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -8206,7 +8206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8892,6 +8892,441 @@
       </c>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>PT-23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>[layout] สองช่อง</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>เปิดแท็บปมเรื่องบนจอคอม</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>ซ้าย = รายการปม (สร้างปมอยู่บนสุด) · ขวา = รายละเอียดปมแรกที่มีเตือน (ไม่มีเตือน = ปมแรก) · สองฝั่งเลื่อนแยกกัน</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>PT-24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>[layout] เลือกปม + URL</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>กดปมอื่นในรายการ แล้วกดย้อนกลับของเบราว์เซอร์</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>URL มี &amp;thread=&lt;id&gt; · ฝั่งขวาเปลี่ยนเป็นปมนั้น แถวในรายการไฮไลต์ · ย้อนกลับได้ปมก่อนหน้า</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>PT-25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>[layout] คำอธิบายไม่ค้าง</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>พิมพ์คำอธิบายปม A ค้างไว้ (ยังไม่คลิกออก) แล้วกดปม B</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>ฝั่งขวาแสดงคำอธิบายของ B ไม่ใช่ข้อความที่พิมพ์ใน A</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>PT-26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>[layout] มือถือ</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>ย่อจอแคบกว่า ~1024px (หรือเปิดบนมือถือ) แล้วกดปม จากนั้นกด "← ปมทั้งหมด"</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>เห็นรายการอย่างเดียว · กดปมแล้วเห็นรายละเอียดอย่างเดียว · ปุ่มกลับพาไปรายการ</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>PT-27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>[layout] สร้างปม</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>พิมพ์ชื่อในช่องสร้างปมแล้วกด "สร้าง"</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>ปมใหม่โผล่ในรายการและถูกเลือกทันที ฝั่งขวาแสดงปมนั้น</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>PT-28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>[layout] ลบปมที่เปิดอยู่</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>กดถังขยะของปมที่กำลังดู</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>ปมหาย หน้าไม่พัง ฝั่งขวาเปลี่ยนไปปมอื่นตามกฎ PT-23 · toast มีปุ่มย้อนกลับ</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>PT-29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>[ความคืบหน้า] คำนวณเอง</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>ปมใหม่ → ผูกฉากหว่าน → ผูกฉากย้ำ → ผูกฉากเฉลย ดูแถบความคืบหน้าทุกขั้น</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>ยังไม่หว่าน → หว่านแล้ว → กำลังสาน → เฉลยครบ (แถบเติมทีละขั้น) · ในรายการซ้ายแสดงคำเดียวกัน</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>PT-30</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>[ความคืบหน้า] เฉลยบางส่วน</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่มีประเด็น 2 ข้อ ติ๊กคลี่ 1 ข้อ (ยังไม่มีฉากเฉลย)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>ความคืบหน้าเป็น "เฉลยบางส่วน"</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>PT-31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>[บั๊กเดิม] ลบฉากเฉลย</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่มีฉากเฉลย ปลดฉากเฉลยนั้นออก</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>ความคืบหน้าถอยกลับ (ไม่ค้าง "เฉลยครบ") · ขึ้นเตือน "ยังไม่มีการเฉลย"</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>PT-32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>[เจตนา] พักไว้</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่ไม่ถูกแตะเกิน 8 บท ตั้งเจตนาเป็น "พักไว้"</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>ป้าย "ไม่ถูกแตะ N บท" หาย · ไม่นับในตัวเลขเตือนของปุ่มสมุดปม · ในรายการขึ้น "· พักไว้"</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>PT-33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>[เจตนา] ปลายเปิด / ทิ้ง</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่ยังไม่เฉลย ตั้งเจตนาเป็น "ตั้งใจค้าง/ปลายเปิด" แล้วลอง "ทิ้งแล้ว"</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>ทั้งสองแบบไม่เตือนว่ายังไม่เฉลย · "ทิ้งแล้ว" แถวในรายการจางลง และไม่มีป้ายเตือนเลย</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>PT-34</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>[เจตนา] ปมเก่า</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>เปิดปมที่เคยตั้งสถานะไว้ก่อนรอบนี้ (หว่านแล้ว/กำลังสาน/เฉลยแล้ว)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>เจตนาแสดงเป็น "ดำเนินอยู่" · ปมที่เคยกด "เฉลยแล้ว" แต่ไม่มีฉากเฉลย ขึ้นเตือน "ยังไม่มีการเฉลย" (ตั้งใจ)</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>PT-35</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>[บทเป้า] เลยเป้า</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>ปมยังไม่เฉลย ตั้ง "ตั้งใจเฉลยภายในบท" เป็นบทที่ไม่ใช่บทสุดท้ายของเรื่อง</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้นป้ายส้ม "เลยบทที่ตั้งใจเฉลยแล้ว" · เปลี่ยนเป็นบทสุดท้าย หรือ "ไม่กำหนด" ป้ายหาย</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>PT-36</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>[บทเป้า] ลบบท</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>ตั้งบทเป้าแล้วลบบทนั้นทิ้ง</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>ปมไม่พัง บทเป้ากลับเป็น "ไม่กำหนด"</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>PT-37</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>[ที่อื่น] รายงานรายตอน + ribbon</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่ตั้ง "ปลายเปิด" และแตะบทที่เปิดรายงานรายตอน / ดูเลนปมบนกระดาน</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>รายงานรายตอนไม่ขึ้น "ปมค้าง" ของปมนี้ · เลนปมไม่ทาบช่วงท้ายว่าค้าง</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Thread journey, richer thread context for AI, AI payoff fairness check
- lib/thread-journey: card-level ordering across the novel; per-thread
  journey (first/payoff card, gaps in cards, other threads in between with
  relation tags, longest silence, clues before payoff per issue)
- Threads tab: journey timeline + clue coverage box with unfair-issue warning
- Scene markdown for AI: Thai progress/intent, tension, thread summary,
  issues and a journey line for threads touching the scene
- New thread-fairness AI feature (qwen3.8-flash via OpenRouter, no Jev):
  guess K=3 before payoff card, judge, continuity checklist; result labelled
  obvious/balanced/twist/unfounded, cached in plot_findings with model/K/hash
- parseCanvasData moved to lib/thread-journey (shared client/server)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -28,6 +28,7 @@
     <sheet name="เส้นเชื่อมสีล้วน v2.10.0" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="ตรวจคำผิด v2.12.0" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="ปมเชิงลึก (ใหม่)" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="เส้นทางปม + AI (ใหม่)" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ผู้ช่วย AI (ใหม่)'!$A$1:$G$19</definedName>
@@ -547,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -752,6 +753,16 @@
       </c>
       <c r="B20" s="10" t="n">
         <v>37</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>เส้นทางปม + AI (ใหม่)</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -9333,6 +9344,762 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TJ-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>[สรุป] จุดแรก/เฉลย</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>เปิดปมที่ผูกการ์ดหว่านและการ์ดเฉลยไว้แล้ว ดูหัวกล่อง "เส้นทางของปม"</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้น "โผล่ครั้งแรก [บท · ฉาก · C0x] · เฉลยที่ [...] · ระยะ N การ์ด · เงียบนานสุด M การ์ด" ตรงกับตำแหน่งการ์ดจริงบนกระดาน</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TJ-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>[ระยะ] นับการ์ด</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่หว่านที่การ์ด C01 ฉาก 1 และย้ำที่ C02 ฉาก 2 (ฉาก 1 มีการ์ด 4 ใบ)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ตัวคั่นระหว่างสองจุดขึ้น "ห่าง 4 การ์ด" · โน้ต (sticky note) ไม่ถูกนับ</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TJ-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>[ระยะ] เรียงตามบท</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่มีจุดในบท 3 และบท 1 (ผูกบท 3 ก่อน)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>จุดบท 1 อยู่บน บท 3 อยู่ล่าง · ระยะเป็นบวก</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TJ-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>[ระหว่างนั้น] ปมอื่น</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>ระหว่างสองจุดของปม A มีการ์ดที่ผูกปม B, C</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ใต้ตัวคั่นขึ้นชิป "ปม B · หว่าน" ฯลฯ · ชี้ค้างเห็นชื่อฉาก+รหัสการ์ด</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TJ-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>[ระหว่างนั้น] ป้าย</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ให้ปม B เป็นปมย่อยของ A และ C "เป็นปมหลอกของ" A</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ชิป B มีป้าย (ปมย่อย) สีฟ้า · ชิป C มีป้าย (ปมหลอกของปมนี้) สีม่วง · ปมไม่เกี่ยวไม่มีป้าย</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TJ-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>[ระหว่างนั้น] เยอะ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ช่วงที่มีปมอื่นเกิน 5 จุด</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>แสดง 5 ชิปแรก + ปุ่ม "+N" กดแล้วเห็นทั้งหมด</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TJ-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>[จุดพิเศษ] ทั้งฉาก</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ผูกปมกับฉากผ่านสมุดปม (ไม่เลือกการ์ด)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>จุดนั้นขึ้นป้าย "ทั้งฉาก" · ระยะนับจากการ์ดแรกของฉาก</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TJ-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>[จุดพิเศษ] ฉากไม่ผูกบท</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ผูกปมกับการ์ดในฉากที่ไม่มีบท</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>จุดนั้นอยู่ท้ายเส้น ป้าย "ไม่ระบุบท" · ตัวคั่นขึ้น "ไม่ทราบระยะ"</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TJ-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>[จุดพิเศษ] การ์ดถูกลบ</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>ลบการ์ดที่ผูกปมบนกระดาน แล้วกลับมาดูปม</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>หน้าไม่พัง · จุดนั้นกลายเป็น "ทั้งฉาก"</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TJ-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>[เบาะแส] นับรายประเด็น</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>ปมมีประเด็น 2 ข้อ · จุดหว่านเลือกประเด็นที่ 1 · มีการ์ดเฉลย</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>กล่อง "เบาะแสก่อนเฉลย" ประเด็น 1 = 1 การ์ด, ประเด็น 2 = 0 การ์ด (สีส้ม)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TJ-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>[เบาะแส] ไม่ยุติธรรม</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ต่อจาก TJ-10 ติ๊กประเด็น 2 ว่าคลี่แล้ว</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้นเตือน ""ประเด็น 2" เฉลยโดยไม่มีเบาะแสมาก่อน" · เลือกประเด็น 2 ให้จุดหว่านแล้วเตือนหาย</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TJ-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>[เบาะแส] ไม่มีประเด็น</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่ไม่มีประเด็นเลย</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>แสดงแถวเดียว "ทั้งปม (ยังไม่แบ่งประเด็น)" นับทุกจุดก่อนเฉลย</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TJ-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>[AI] ไฟล์ส่งออกฉาก</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>บนกระดานฉากที่มีปมผ่าน กดส่งออก/คัดลอก Markdown ของฉาก</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ตารางปมมีคอลัมน์ ความคืบหน้า / เจตนาผู้เขียน / ความตึงในฉากนี้ เป็นคำไทย · มีหัว ปม "...": คืออะไร + ประเด็น ([x]/[ ]) + "← ฉากนี้ขยับประเด็นนี้"</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TJ-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>[AI] สรุปฉาก</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>กดสรุปฉาก (AI) ในฉากที่มีปมพร้อมคำอธิบาย</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>สรุปใช้ได้ปกติ ไม่ error · (ถ้าดูได้) เนื้อหาสะท้อนประเด็นของปม</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TJ-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>[AI] ปมไม่ผ่านฉาก</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่มีคำอธิบายแต่ไม่ผูกฉากนี้ แล้วส่งออก Markdown ของฉากนี้</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>ไม่มีคำอธิบายของปมนั้นใน Markdown (มีแค่ชื่อในหัวข้อ "ปมที่ยังไม่เฉลย" ถ้ายังค้าง)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TF-01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] ไม่มีเฉลย</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>เปิดปมที่ยังไม่มีการ์ดเฉลย</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>ส่วน "ตรวจการเฉลย (AI)" ขึ้น "ต้องผูกการ์ดเฉลยก่อนถึงจะตรวจได้" ไม่มีปุ่ม</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TF-02</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] ตรวจครั้งแรก</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่มีหว่าน+เฉลย กด "ตรวจการเฉลย" (เช่น "เสียงปริศนาที่พระเอกได้ยิน")</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>ปุ่มขึ้น "กำลังตรวจ…" แล้วได้ป้าย 1 ใน 4 (ชัดเจน/พอดี/หักมุม/เบาะแสไม่พอ) · "ทายต่อ 3 ข้อ ถึงเฉลย N ข้อ" พร้อมคำทาย ✓/✗ · เช็คลิสต์ 3 ข้อ · บรรทัดล่างมี qwen/qwen3.8-flash · K=3 · เวลา</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TF-03</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] ผลถูกเก็บ</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>ต่อจาก TF-02 สลับไปปมอื่นแล้วกลับมา / รีเฟรชหน้า</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>ผลเดิมโผล่ทันทีโดยไม่ต้องกดใหม่ · ไม่มีป้าย "ผลเก่า"</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TF-04</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] ผลเก่า</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>แก้เนื้อการ์ดหว่านของปมบนกระดาน แล้วกลับมาดูปม</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้นป้าย "ผลเก่า — การ์ดเปลี่ยนแล้ว"</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TF-05</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] ไม่เปลี่ยนไม่เรียกซ้ำ</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>กด "ตรวจใหม่" สองครั้งติดกัน</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>ทั้งสองครั้งเรียก AI จริง (ตรวจใหม่บังคับ) · ดู log การใช้ AI ฟีเจอร์ "ตรวจการเฉลยปม" เพิ่มครั้งละ 3 แถว</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TF-06</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] ไม่มีคำอธิบาย</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่ไม่มีคำอธิบาย กดตรวจ</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>ตรวจได้ · ขึ้นป้าย "ใส่คำอธิบายปมแล้วผลจะแม่นขึ้น"</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TF-07</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] การ์ดเฉลยสั้น</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>ปมที่การ์ดเฉลยมีแค่ชื่อ ไม่มีเนื้อ กดตรวจ</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้นป้าย "การ์ดเฉลยสั้น ผลเชื่อได้น้อย"</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TF-08</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] quota/ปิดฟีเจอร์</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>ปิดฟีเจอร์ "ตรวจการเฉลยปม" ในหน้า AI Control แล้วกดตรวจ</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>ขึ้น toast error ไม่พัง ไม่บันทึกผลใหม่</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TF-09</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>[AI ตรวจเฉลย] สมเหตุสมผล</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ลองกับปมที่ตั้งใจให้เดาง่าย (เบาะแสชัด) เทียบปมที่เฉลยแบบโผล่มาเฉยๆ</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>ปมเดาง่ายมีแนวโน้มได้ "ชัดเจน"/"พอดี" · ปมโผล่เฉยๆ มีแนวโน้มได้ "เบาะแสไม่พอ" (K=3 แกว่งได้ ดูแนวโน้มหลายครั้ง)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Thread groups: combined journey lanes + open-children warning
- groupJourney: root thread plus all descendants as lanes on one card axis,
  with descendants paid/total
- Thread detail shows the group lanes when the thread has sub-threads
- New network warning: parent has a payoff while a descendant is still open

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="B21" s="10" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -9350,7 +9350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10094,6 +10094,151 @@
       </c>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TG-01</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>[กลุ่ม] เส้นทางรวม</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>ตั้งปม B, C ให้อยู่ใต้ปม A (และ D ใต้ B) แล้วเปิดปม A</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>มีกล่อง "เส้นทางรวมของกลุ่ม · ปมย่อยเฉลยแล้ว x/3" · เลน A บนสุด ตามด้วย B, D (เยื้อง ↳), C · จุดหว่าน/ย้ำเป็นวงกลม เฉลยเป็นเพชร อยู่ตำแหน่งตรงกับลำดับการ์ด</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TG-02</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>[กลุ่ม] เส้นประ</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>ปมย่อยที่ยังไม่เฉลย</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>เลนนั้นเป็นเส้นประ · ปมที่เฉลยแล้วเป็นเส้นทึบ</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TG-03</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>[กลุ่ม] กดเปิดปมย่อย</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>กดชื่อเลนปมย่อย</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>เปิดรายละเอียดปมย่อยนั้น URL เปลี่ยน ?thread=</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TG-04</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>[กลุ่ม] ปมไม่มีลูก</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>เปิดปมที่ไม่มีปมย่อย</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>ไม่มีกล่องเส้นทางรวมของกลุ่ม</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TG-05</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>[เตือน] ปมใหญ่เฉลยแต่ลูกค้าง</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>ผูกการ์ดเฉลยให้ปม A ขณะที่ D (หลาน) ยังไม่เฉลย</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>A ขึ้นป้าย "เฉลยแล้ว แต่ปมย่อยยังค้าง 1 ปม" · ตัวเลขเตือนบนแท็บเพิ่ม · ตั้ง D เป็น "ทิ้งแล้ว" หรือผูกเฉลยให้ D แล้วป้ายหาย</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Thread undo restores the full thread
- Snapshot now keeps status, summary, parent, target chapter, issues,
  child ids, links both ways, and each beat's card/issue/tension
- Restore recreates issues (old→new id map), re-links children and links;
  reports "กู้คืนได้ไม่ครบ" for parts that no longer can be restored
- Beat undo keeps card/issue/tension too; old localStorage entries still read

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21">
@@ -8217,7 +8217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8883,7 +8883,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>[ข้อจำกัด] ลบแล้วย้อนกลับ</t>
+          <t>[ย้อนกลับ] ลบแล้วกู้คืน</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -8893,12 +8893,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ปมกลับมาพร้อมฉากที่ผูก แต่คำอธิบาย/ประเด็น/ความสัมพันธ์/ความตึงหาย (ข้อจำกัดที่รู้แล้ว task.md ข้อ 18)</t>
+          <t>ปมกลับมาครบ: คำอธิบาย ประเด็น (สถานะคลี่เดิม) เจตนา บทเป้า ปมแม่ ปมย่อยกลับมาอยู่ใต้ ความสัมพันธ์ทั้งสองทาง และแต่ละจุดผูกการ์ด/ประเด็น/ความตึงเดิม · ผลตรวจ AI ไม่กลับ (ต้องกดตรวจใหม่)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>ต่ำ</t>
+          <t>สูง</t>
         </is>
       </c>
       <c r="F23" s="2" t="n"/>
@@ -9338,6 +9338,35 @@
       </c>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>PT-38</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>[ย้อนกลับ] กู้ได้บางส่วน</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>ลบปม A (ที่มีความสัมพันธ์กับปม B) → ลบปม B → กด "ย้อนกลับ" ของปม A จากเมนูกู้คืน</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>ปม A กลับมา · ขึ้น toast แดง "กู้คืนได้ไม่ครบ: ความสัมพันธ์" · หน้าไม่พัง</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>